<commit_message>
Update HOTAS Switch and Button - Quick Reference - BASIC - T16000.xlsx
</commit_message>
<xml_diff>
--- a/MapFiles/HOTAS Switch and Button - Quick Reference - BASIC - T16000.xlsx
+++ b/MapFiles/HOTAS Switch and Button - Quick Reference - BASIC - T16000.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Users\Den\OneDrive\Personal\Thrustmaster\TARGET\Clicker\Development\ED_Enhanced_T16000\MapFiles\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1AD1550B-2F31-47F3-8F08-4FC49DB37B7E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{24A39E6F-7AA7-4F82-9A87-FCFAE880FA2E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="18495" yWindow="705" windowWidth="19725" windowHeight="20235" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -278,14 +278,37 @@
     <t>TFRPHA_LEFT</t>
   </si>
   <si>
-    <t>HOTAS - Quick reference -  BASIC - T16000 &amp; TWCS Throttle</t>
+    <r>
+      <t xml:space="preserve">HOTAS - Quick reference - </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> BASIC</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> - T16000 &amp; TWCS Throttle</t>
+    </r>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -295,6 +318,14 @@
     </font>
     <font>
       <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -903,7 +934,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="91">
+  <cellXfs count="81">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1028,6 +1059,60 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="40" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="32" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="34" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="34" xfId="0" quotePrefix="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" quotePrefix="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="41" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1090,90 +1175,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="29" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="40" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="32" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="34" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="34" xfId="0" quotePrefix="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" quotePrefix="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="41" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1481,17 +1482,17 @@
   <sheetData>
     <row r="1" spans="2:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="2:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="55" t="s">
+      <c r="B2" s="73" t="s">
         <v>80</v>
       </c>
-      <c r="C2" s="56"/>
-      <c r="D2" s="56"/>
-      <c r="E2" s="56"/>
-      <c r="F2" s="56"/>
-      <c r="G2" s="56"/>
-      <c r="H2" s="56"/>
-      <c r="I2" s="56"/>
-      <c r="J2" s="57"/>
+      <c r="C2" s="74"/>
+      <c r="D2" s="74"/>
+      <c r="E2" s="74"/>
+      <c r="F2" s="74"/>
+      <c r="G2" s="74"/>
+      <c r="H2" s="74"/>
+      <c r="I2" s="74"/>
+      <c r="J2" s="75"/>
       <c r="K2"/>
       <c r="L2"/>
       <c r="M2"/>
@@ -1506,18 +1507,18 @@
       <c r="O3"/>
     </row>
     <row r="4" spans="2:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B4" s="48" t="s">
+      <c r="B4" s="66" t="s">
         <v>9</v>
       </c>
-      <c r="C4" s="49"/>
-      <c r="D4" s="49"/>
-      <c r="E4" s="50"/>
-      <c r="G4" s="48" t="s">
+      <c r="C4" s="67"/>
+      <c r="D4" s="67"/>
+      <c r="E4" s="68"/>
+      <c r="G4" s="66" t="s">
         <v>8</v>
       </c>
-      <c r="H4" s="49"/>
-      <c r="I4" s="49"/>
-      <c r="J4" s="50"/>
+      <c r="H4" s="67"/>
+      <c r="I4" s="67"/>
+      <c r="J4" s="68"/>
       <c r="K4"/>
       <c r="L4"/>
       <c r="M4"/>
@@ -1568,7 +1569,7 @@
       <c r="C7" s="27" t="s">
         <v>63</v>
       </c>
-      <c r="D7" s="90" t="s">
+      <c r="D7" s="59" t="s">
         <v>54</v>
       </c>
       <c r="E7" s="17" t="s">
@@ -1580,7 +1581,7 @@
       <c r="H7" s="27" t="s">
         <v>63</v>
       </c>
-      <c r="I7" s="90" t="s">
+      <c r="I7" s="59" t="s">
         <v>57</v>
       </c>
       <c r="J7" s="17" t="s">
@@ -1598,7 +1599,7 @@
       <c r="C8" s="31" t="s">
         <v>63</v>
       </c>
-      <c r="D8" s="65" t="s">
+      <c r="D8" s="2" t="s">
         <v>55</v>
       </c>
       <c r="E8" s="3" t="s">
@@ -1610,7 +1611,7 @@
       <c r="H8" s="31" t="s">
         <v>63</v>
       </c>
-      <c r="I8" s="65" t="s">
+      <c r="I8" s="2" t="s">
         <v>56</v>
       </c>
       <c r="J8" s="3" t="s">
@@ -1628,7 +1629,7 @@
       <c r="C9" s="31" t="s">
         <v>63</v>
       </c>
-      <c r="D9" s="65" t="s">
+      <c r="D9" s="2" t="s">
         <v>56</v>
       </c>
       <c r="E9" s="3" t="s">
@@ -1640,7 +1641,7 @@
       <c r="H9" s="31" t="s">
         <v>63</v>
       </c>
-      <c r="I9" s="65" t="s">
+      <c r="I9" s="2" t="s">
         <v>58</v>
       </c>
       <c r="J9" s="3" t="s">
@@ -1668,7 +1669,7 @@
       <c r="H10" s="31" t="s">
         <v>63</v>
       </c>
-      <c r="I10" s="65" t="s">
+      <c r="I10" s="2" t="s">
         <v>59</v>
       </c>
       <c r="J10" s="3" t="s">
@@ -1686,7 +1687,7 @@
       <c r="H11" s="32" t="s">
         <v>63</v>
       </c>
-      <c r="I11" s="72" t="s">
+      <c r="I11" s="4" t="s">
         <v>69</v>
       </c>
       <c r="J11" s="5" t="s">
@@ -1726,873 +1727,858 @@
     </row>
     <row r="14" spans="2:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="15" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B15" s="58" t="s">
+      <c r="B15" s="76" t="s">
         <v>11</v>
       </c>
       <c r="C15" s="9" t="s">
         <v>61</v>
       </c>
-      <c r="D15" s="63"/>
-      <c r="E15" s="64"/>
-      <c r="G15" s="47" t="s">
+      <c r="D15" s="9"/>
+      <c r="E15" s="42"/>
+      <c r="G15" s="65" t="s">
         <v>26</v>
       </c>
       <c r="H15" s="9" t="s">
         <v>61</v>
       </c>
-      <c r="I15" s="63"/>
-      <c r="J15" s="64"/>
+      <c r="I15" s="9"/>
+      <c r="J15" s="42"/>
       <c r="L15" s="8"/>
     </row>
     <row r="16" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B16" s="51"/>
+      <c r="B16" s="69"/>
       <c r="C16" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="D16" s="65"/>
-      <c r="E16" s="66"/>
-      <c r="G16" s="43"/>
+      <c r="D16" s="2"/>
+      <c r="E16" s="3"/>
+      <c r="G16" s="61"/>
       <c r="H16" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="I16" s="80"/>
-      <c r="J16" s="66"/>
+      <c r="I16" s="50"/>
+      <c r="J16" s="3"/>
       <c r="L16" s="8"/>
     </row>
     <row r="17" spans="2:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B17" s="54"/>
+      <c r="B17" s="72"/>
       <c r="C17" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="D17" s="67"/>
-      <c r="E17" s="68"/>
-      <c r="G17" s="44"/>
+      <c r="D17" s="43"/>
+      <c r="E17" s="5"/>
+      <c r="G17" s="62"/>
       <c r="H17" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="I17" s="81"/>
-      <c r="J17" s="76"/>
+      <c r="I17" s="51"/>
+      <c r="J17" s="47"/>
       <c r="L17" s="8"/>
     </row>
     <row r="18" spans="2:16" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="D18" s="69"/>
-      <c r="E18" s="69"/>
       <c r="G18" s="26" t="s">
         <v>27</v>
       </c>
       <c r="H18" s="27" t="s">
         <v>63</v>
       </c>
-      <c r="I18" s="82"/>
-      <c r="J18" s="83"/>
+      <c r="I18" s="52"/>
+      <c r="J18" s="53"/>
     </row>
     <row r="19" spans="2:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B19" s="58" t="s">
+      <c r="B19" s="76" t="s">
         <v>10</v>
       </c>
       <c r="C19" s="9" t="s">
         <v>61</v>
       </c>
-      <c r="D19" s="63"/>
-      <c r="E19" s="64"/>
+      <c r="D19" s="9"/>
+      <c r="E19" s="42"/>
       <c r="G19" s="28" t="s">
         <v>28</v>
       </c>
       <c r="H19" s="29" t="s">
         <v>63</v>
       </c>
-      <c r="I19" s="81"/>
-      <c r="J19" s="76"/>
+      <c r="I19" s="51"/>
+      <c r="J19" s="47"/>
       <c r="L19" s="8"/>
     </row>
     <row r="20" spans="2:16" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="B20" s="51"/>
+      <c r="B20" s="69"/>
       <c r="C20" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="D20" s="65"/>
-      <c r="E20" s="66"/>
-      <c r="G20" s="59" t="s">
+      <c r="D20" s="2"/>
+      <c r="E20" s="3"/>
+      <c r="G20" s="77" t="s">
         <v>29</v>
       </c>
       <c r="H20" s="21" t="s">
         <v>61</v>
       </c>
-      <c r="I20" s="82"/>
-      <c r="J20" s="77"/>
+      <c r="I20" s="52"/>
+      <c r="J20" s="48"/>
       <c r="L20" s="8"/>
     </row>
     <row r="21" spans="2:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B21" s="54"/>
+      <c r="B21" s="72"/>
       <c r="C21" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="D21" s="67"/>
-      <c r="E21" s="68"/>
-      <c r="G21" s="60"/>
+      <c r="D21" s="43"/>
+      <c r="E21" s="5"/>
+      <c r="G21" s="78"/>
       <c r="H21" s="11" t="s">
         <v>60</v>
       </c>
-      <c r="I21" s="65"/>
-      <c r="J21" s="66"/>
+      <c r="I21" s="2"/>
+      <c r="J21" s="3"/>
     </row>
     <row r="22" spans="2:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B22" s="8"/>
-      <c r="D22" s="69"/>
-      <c r="E22" s="69"/>
-      <c r="G22" s="61"/>
+      <c r="G22" s="79"/>
       <c r="H22" s="24" t="s">
         <v>62</v>
       </c>
-      <c r="I22" s="81"/>
-      <c r="J22" s="76"/>
+      <c r="I22" s="51"/>
+      <c r="J22" s="47"/>
       <c r="L22" s="8"/>
     </row>
     <row r="23" spans="2:16" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="B23" s="58" t="s">
+      <c r="B23" s="76" t="s">
         <v>12</v>
       </c>
       <c r="C23" s="9" t="s">
         <v>61</v>
       </c>
-      <c r="D23" s="63"/>
-      <c r="E23" s="64"/>
-      <c r="G23" s="60" t="s">
+      <c r="D23" s="9"/>
+      <c r="E23" s="42"/>
+      <c r="G23" s="78" t="s">
         <v>30</v>
       </c>
       <c r="H23" s="25" t="s">
         <v>61</v>
       </c>
-      <c r="I23" s="84"/>
-      <c r="J23" s="71"/>
+      <c r="I23" s="54"/>
+      <c r="J23" s="44"/>
       <c r="L23" s="8"/>
     </row>
     <row r="24" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B24" s="51"/>
+      <c r="B24" s="69"/>
       <c r="C24" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="D24" s="70"/>
-      <c r="E24" s="71"/>
-      <c r="G24" s="60"/>
+      <c r="D24" s="13"/>
+      <c r="E24" s="44"/>
+      <c r="G24" s="78"/>
       <c r="H24" s="11" t="s">
         <v>60</v>
       </c>
-      <c r="I24" s="65"/>
-      <c r="J24" s="85"/>
+      <c r="I24" s="2"/>
+      <c r="J24" s="55"/>
     </row>
     <row r="25" spans="2:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B25" s="54"/>
+      <c r="B25" s="72"/>
       <c r="C25" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="D25" s="72"/>
-      <c r="E25" s="68"/>
-      <c r="G25" s="62"/>
+      <c r="D25" s="4"/>
+      <c r="E25" s="5"/>
+      <c r="G25" s="80"/>
       <c r="H25" s="12" t="s">
         <v>62</v>
       </c>
-      <c r="I25" s="81"/>
-      <c r="J25" s="68"/>
+      <c r="I25" s="51"/>
+      <c r="J25" s="5"/>
       <c r="L25" s="8"/>
     </row>
     <row r="26" spans="2:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B26" s="8"/>
-      <c r="D26" s="69"/>
-      <c r="E26" s="69"/>
-      <c r="I26" s="86"/>
-      <c r="J26" s="69"/>
+      <c r="I26" s="22"/>
     </row>
     <row r="27" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B27" s="58" t="s">
+      <c r="B27" s="76" t="s">
         <v>13</v>
       </c>
       <c r="C27" s="9" t="s">
         <v>61</v>
       </c>
-      <c r="D27" s="63"/>
-      <c r="E27" s="64"/>
-      <c r="G27" s="58" t="s">
+      <c r="D27" s="9"/>
+      <c r="E27" s="42"/>
+      <c r="G27" s="76" t="s">
         <v>31</v>
       </c>
       <c r="H27" s="9" t="s">
         <v>61</v>
       </c>
-      <c r="I27" s="87"/>
-      <c r="J27" s="64"/>
+      <c r="I27" s="56"/>
+      <c r="J27" s="42"/>
       <c r="L27" s="8"/>
     </row>
     <row r="28" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B28" s="51"/>
+      <c r="B28" s="69"/>
       <c r="C28" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="D28" s="73"/>
-      <c r="E28" s="66"/>
-      <c r="G28" s="51"/>
+      <c r="D28" s="45"/>
+      <c r="E28" s="3"/>
+      <c r="G28" s="69"/>
       <c r="H28" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="I28" s="80"/>
-      <c r="J28" s="66"/>
+      <c r="I28" s="50"/>
+      <c r="J28" s="3"/>
     </row>
     <row r="29" spans="2:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B29" s="54"/>
+      <c r="B29" s="72"/>
       <c r="C29" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="D29" s="72"/>
-      <c r="E29" s="68"/>
-      <c r="G29" s="54"/>
+      <c r="D29" s="4"/>
+      <c r="E29" s="5"/>
+      <c r="G29" s="72"/>
       <c r="H29" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="I29" s="88"/>
-      <c r="J29" s="68"/>
+      <c r="I29" s="57"/>
+      <c r="J29" s="5"/>
       <c r="L29" s="8"/>
     </row>
     <row r="30" spans="2:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="D30" s="69"/>
-      <c r="E30" s="69"/>
       <c r="G30" s="7"/>
-      <c r="I30" s="86"/>
-      <c r="J30" s="69"/>
+      <c r="I30" s="22"/>
       <c r="L30" s="8"/>
     </row>
     <row r="31" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B31" s="58" t="s">
+      <c r="B31" s="76" t="s">
         <v>0</v>
       </c>
       <c r="C31" s="9" t="s">
         <v>61</v>
       </c>
-      <c r="D31" s="63"/>
-      <c r="E31" s="64"/>
-      <c r="G31" s="47" t="s">
+      <c r="D31" s="9"/>
+      <c r="E31" s="42"/>
+      <c r="G31" s="65" t="s">
         <v>32</v>
       </c>
       <c r="H31" s="9" t="s">
         <v>61</v>
       </c>
-      <c r="I31" s="63"/>
-      <c r="J31" s="64"/>
+      <c r="I31" s="9"/>
+      <c r="J31" s="42"/>
       <c r="P31" s="22"/>
     </row>
     <row r="32" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B32" s="51"/>
+      <c r="B32" s="69"/>
       <c r="C32" s="13" t="s">
         <v>60</v>
       </c>
-      <c r="D32" s="65"/>
-      <c r="E32" s="71"/>
-      <c r="G32" s="43"/>
+      <c r="D32" s="2"/>
+      <c r="E32" s="44"/>
+      <c r="G32" s="61"/>
       <c r="H32" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="I32" s="65"/>
-      <c r="J32" s="66"/>
+      <c r="I32" s="2"/>
+      <c r="J32" s="3"/>
       <c r="L32" s="8"/>
       <c r="P32" s="22"/>
     </row>
     <row r="33" spans="2:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B33" s="52"/>
+      <c r="B33" s="70"/>
       <c r="C33" s="23" t="s">
         <v>62</v>
       </c>
-      <c r="D33" s="74"/>
-      <c r="E33" s="75"/>
-      <c r="G33" s="44"/>
+      <c r="D33" s="6"/>
+      <c r="E33" s="46"/>
+      <c r="G33" s="62"/>
       <c r="H33" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="I33" s="74"/>
-      <c r="J33" s="76"/>
+      <c r="I33" s="6"/>
+      <c r="J33" s="47"/>
       <c r="L33" s="8"/>
       <c r="P33" s="22"/>
     </row>
     <row r="34" spans="2:17" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="B34" s="51" t="s">
+      <c r="B34" s="69" t="s">
         <v>1</v>
       </c>
       <c r="C34" s="13" t="s">
         <v>61</v>
       </c>
-      <c r="D34" s="70"/>
-      <c r="E34" s="71"/>
-      <c r="G34" s="42" t="s">
+      <c r="D34" s="13"/>
+      <c r="E34" s="44"/>
+      <c r="G34" s="60" t="s">
         <v>33</v>
       </c>
       <c r="H34" s="21" t="s">
         <v>61</v>
       </c>
-      <c r="I34" s="79"/>
-      <c r="J34" s="77"/>
+      <c r="I34" s="21"/>
+      <c r="J34" s="48"/>
       <c r="P34" s="22"/>
     </row>
     <row r="35" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B35" s="51"/>
+      <c r="B35" s="69"/>
       <c r="C35" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="D35" s="65"/>
-      <c r="E35" s="66"/>
-      <c r="G35" s="43"/>
+      <c r="D35" s="2"/>
+      <c r="E35" s="3"/>
+      <c r="G35" s="61"/>
       <c r="H35" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="I35" s="65"/>
-      <c r="J35" s="66"/>
+      <c r="I35" s="2"/>
+      <c r="J35" s="3"/>
       <c r="L35" s="8"/>
       <c r="P35" s="22"/>
     </row>
     <row r="36" spans="2:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B36" s="52"/>
+      <c r="B36" s="70"/>
       <c r="C36" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="D36" s="74"/>
-      <c r="E36" s="76"/>
-      <c r="G36" s="44"/>
+      <c r="D36" s="6"/>
+      <c r="E36" s="47"/>
+      <c r="G36" s="62"/>
       <c r="H36" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="I36" s="74"/>
-      <c r="J36" s="76"/>
+      <c r="I36" s="6"/>
+      <c r="J36" s="47"/>
       <c r="L36" s="8"/>
       <c r="P36" s="22"/>
       <c r="Q36" s="7"/>
     </row>
     <row r="37" spans="2:17" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="B37" s="53" t="s">
+      <c r="B37" s="71" t="s">
         <v>2</v>
       </c>
       <c r="C37" s="21" t="s">
         <v>61</v>
       </c>
-      <c r="D37" s="70"/>
-      <c r="E37" s="77"/>
-      <c r="G37" s="42" t="s">
+      <c r="D37" s="13"/>
+      <c r="E37" s="48"/>
+      <c r="G37" s="60" t="s">
         <v>34</v>
       </c>
       <c r="H37" s="21" t="s">
         <v>61</v>
       </c>
-      <c r="I37" s="70"/>
-      <c r="J37" s="77"/>
+      <c r="I37" s="13"/>
+      <c r="J37" s="48"/>
       <c r="P37" s="22"/>
       <c r="Q37" s="7"/>
     </row>
     <row r="38" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B38" s="51"/>
+      <c r="B38" s="69"/>
       <c r="C38" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="D38" s="65"/>
-      <c r="E38" s="66"/>
-      <c r="G38" s="43"/>
+      <c r="D38" s="2"/>
+      <c r="E38" s="3"/>
+      <c r="G38" s="61"/>
       <c r="H38" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="I38" s="65"/>
-      <c r="J38" s="66"/>
+      <c r="I38" s="2"/>
+      <c r="J38" s="3"/>
       <c r="L38" s="8"/>
       <c r="P38" s="22"/>
       <c r="Q38" s="7"/>
     </row>
     <row r="39" spans="2:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B39" s="52"/>
+      <c r="B39" s="70"/>
       <c r="C39" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="D39" s="74"/>
-      <c r="E39" s="75"/>
-      <c r="G39" s="44"/>
+      <c r="D39" s="6"/>
+      <c r="E39" s="46"/>
+      <c r="G39" s="62"/>
       <c r="H39" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="I39" s="74"/>
-      <c r="J39" s="75"/>
+      <c r="I39" s="6"/>
+      <c r="J39" s="46"/>
       <c r="L39" s="8"/>
       <c r="P39" s="22"/>
       <c r="Q39" s="7"/>
     </row>
     <row r="40" spans="2:17" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="B40" s="53" t="s">
+      <c r="B40" s="71" t="s">
         <v>3</v>
       </c>
       <c r="C40" s="21" t="s">
         <v>61</v>
       </c>
-      <c r="D40" s="70"/>
-      <c r="E40" s="66"/>
-      <c r="G40" s="45" t="s">
+      <c r="D40" s="13"/>
+      <c r="E40" s="3"/>
+      <c r="G40" s="63" t="s">
         <v>35</v>
       </c>
       <c r="H40" s="13" t="s">
         <v>61</v>
       </c>
-      <c r="I40" s="70"/>
-      <c r="J40" s="71"/>
+      <c r="I40" s="13"/>
+      <c r="J40" s="44"/>
       <c r="P40" s="22"/>
     </row>
     <row r="41" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B41" s="51"/>
+      <c r="B41" s="69"/>
       <c r="C41" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="D41" s="65"/>
-      <c r="E41" s="66"/>
-      <c r="G41" s="43"/>
+      <c r="D41" s="2"/>
+      <c r="E41" s="3"/>
+      <c r="G41" s="61"/>
       <c r="H41" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="I41" s="65"/>
-      <c r="J41" s="66"/>
+      <c r="I41" s="2"/>
+      <c r="J41" s="3"/>
       <c r="L41" s="8"/>
       <c r="P41" s="22"/>
     </row>
     <row r="42" spans="2:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B42" s="54"/>
+      <c r="B42" s="72"/>
       <c r="C42" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="D42" s="72"/>
-      <c r="E42" s="78"/>
-      <c r="G42" s="46"/>
+      <c r="D42" s="4"/>
+      <c r="E42" s="49"/>
+      <c r="G42" s="64"/>
       <c r="H42" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="I42" s="72"/>
-      <c r="J42" s="68"/>
+      <c r="I42" s="4"/>
+      <c r="J42" s="5"/>
       <c r="L42" s="8"/>
       <c r="P42" s="22"/>
     </row>
     <row r="43" spans="2:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="D43" s="69"/>
-      <c r="E43" s="69"/>
       <c r="G43" s="8"/>
-      <c r="I43" s="86"/>
-      <c r="J43" s="69"/>
+      <c r="I43" s="22"/>
       <c r="P43" s="22"/>
     </row>
     <row r="44" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B44" s="47" t="s">
+      <c r="B44" s="65" t="s">
         <v>14</v>
       </c>
       <c r="C44" s="9" t="s">
         <v>61</v>
       </c>
-      <c r="D44" s="63"/>
-      <c r="E44" s="64"/>
-      <c r="G44" s="47" t="s">
+      <c r="D44" s="9"/>
+      <c r="E44" s="42"/>
+      <c r="G44" s="65" t="s">
         <v>36</v>
       </c>
       <c r="H44" s="9" t="s">
         <v>61</v>
       </c>
-      <c r="I44" s="63"/>
-      <c r="J44" s="64"/>
+      <c r="I44" s="9"/>
+      <c r="J44" s="42"/>
       <c r="L44" s="8"/>
       <c r="P44" s="22"/>
     </row>
     <row r="45" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B45" s="43"/>
+      <c r="B45" s="61"/>
       <c r="C45" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="D45" s="65"/>
-      <c r="E45" s="66"/>
-      <c r="G45" s="43"/>
+      <c r="D45" s="2"/>
+      <c r="E45" s="3"/>
+      <c r="G45" s="61"/>
       <c r="H45" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="I45" s="65"/>
-      <c r="J45" s="66"/>
+      <c r="I45" s="2"/>
+      <c r="J45" s="3"/>
       <c r="L45" s="8"/>
     </row>
     <row r="46" spans="2:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B46" s="44"/>
+      <c r="B46" s="62"/>
       <c r="C46" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="D46" s="74"/>
-      <c r="E46" s="76"/>
-      <c r="G46" s="44"/>
+      <c r="D46" s="6"/>
+      <c r="E46" s="47"/>
+      <c r="G46" s="62"/>
       <c r="H46" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="I46" s="74"/>
-      <c r="J46" s="76"/>
+      <c r="I46" s="6"/>
+      <c r="J46" s="47"/>
     </row>
     <row r="47" spans="2:17" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="B47" s="42" t="s">
+      <c r="B47" s="60" t="s">
         <v>15</v>
       </c>
       <c r="C47" s="21" t="s">
         <v>61</v>
       </c>
-      <c r="D47" s="65"/>
-      <c r="E47" s="77"/>
-      <c r="G47" s="42" t="s">
+      <c r="D47" s="2"/>
+      <c r="E47" s="48"/>
+      <c r="G47" s="60" t="s">
         <v>37</v>
       </c>
       <c r="H47" s="21" t="s">
         <v>61</v>
       </c>
-      <c r="I47" s="79"/>
-      <c r="J47" s="77"/>
+      <c r="I47" s="21"/>
+      <c r="J47" s="48"/>
       <c r="L47" s="8"/>
     </row>
     <row r="48" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B48" s="43"/>
+      <c r="B48" s="61"/>
       <c r="C48" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="D48" s="65"/>
-      <c r="E48" s="66"/>
-      <c r="G48" s="43"/>
+      <c r="D48" s="2"/>
+      <c r="E48" s="3"/>
+      <c r="G48" s="61"/>
       <c r="H48" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="I48" s="65"/>
-      <c r="J48" s="66"/>
+      <c r="I48" s="2"/>
+      <c r="J48" s="3"/>
       <c r="L48" s="8"/>
     </row>
     <row r="49" spans="2:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B49" s="44"/>
+      <c r="B49" s="62"/>
       <c r="C49" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="D49" s="74"/>
-      <c r="E49" s="76"/>
-      <c r="G49" s="44"/>
+      <c r="D49" s="6"/>
+      <c r="E49" s="47"/>
+      <c r="G49" s="62"/>
       <c r="H49" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="I49" s="74"/>
-      <c r="J49" s="76"/>
+      <c r="I49" s="6"/>
+      <c r="J49" s="47"/>
     </row>
     <row r="50" spans="2:10" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="B50" s="42" t="s">
+      <c r="B50" s="60" t="s">
         <v>16</v>
       </c>
       <c r="C50" s="21" t="s">
         <v>61</v>
       </c>
-      <c r="D50" s="79"/>
-      <c r="E50" s="77"/>
-      <c r="G50" s="42" t="s">
+      <c r="D50" s="21"/>
+      <c r="E50" s="48"/>
+      <c r="G50" s="60" t="s">
         <v>38</v>
       </c>
       <c r="H50" s="21" t="s">
         <v>61</v>
       </c>
-      <c r="I50" s="79"/>
-      <c r="J50" s="77"/>
+      <c r="I50" s="21"/>
+      <c r="J50" s="48"/>
     </row>
     <row r="51" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B51" s="43"/>
+      <c r="B51" s="61"/>
       <c r="C51" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="D51" s="65"/>
-      <c r="E51" s="66"/>
-      <c r="G51" s="43"/>
+      <c r="D51" s="2"/>
+      <c r="E51" s="3"/>
+      <c r="G51" s="61"/>
       <c r="H51" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="I51" s="65"/>
-      <c r="J51" s="66"/>
+      <c r="I51" s="2"/>
+      <c r="J51" s="3"/>
     </row>
     <row r="52" spans="2:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B52" s="44"/>
+      <c r="B52" s="62"/>
       <c r="C52" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="D52" s="74"/>
-      <c r="E52" s="76"/>
-      <c r="G52" s="44"/>
+      <c r="D52" s="6"/>
+      <c r="E52" s="47"/>
+      <c r="G52" s="62"/>
       <c r="H52" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="I52" s="74"/>
-      <c r="J52" s="76"/>
+      <c r="I52" s="6"/>
+      <c r="J52" s="47"/>
     </row>
     <row r="53" spans="2:10" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="B53" s="42" t="s">
+      <c r="B53" s="60" t="s">
         <v>17</v>
       </c>
       <c r="C53" s="21" t="s">
         <v>61</v>
       </c>
-      <c r="D53" s="79"/>
-      <c r="E53" s="77"/>
-      <c r="G53" s="45" t="s">
+      <c r="D53" s="21"/>
+      <c r="E53" s="48"/>
+      <c r="G53" s="63" t="s">
         <v>39</v>
       </c>
       <c r="H53" s="13" t="s">
         <v>61</v>
       </c>
-      <c r="I53" s="70"/>
-      <c r="J53" s="71"/>
+      <c r="I53" s="13"/>
+      <c r="J53" s="44"/>
     </row>
     <row r="54" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B54" s="43"/>
+      <c r="B54" s="61"/>
       <c r="C54" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="D54" s="65"/>
-      <c r="E54" s="66"/>
-      <c r="G54" s="43"/>
+      <c r="D54" s="2"/>
+      <c r="E54" s="3"/>
+      <c r="G54" s="61"/>
       <c r="H54" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="I54" s="65"/>
-      <c r="J54" s="66"/>
+      <c r="I54" s="2"/>
+      <c r="J54" s="3"/>
     </row>
     <row r="55" spans="2:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B55" s="44"/>
+      <c r="B55" s="62"/>
       <c r="C55" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="D55" s="74"/>
-      <c r="E55" s="76"/>
-      <c r="G55" s="46"/>
+      <c r="D55" s="6"/>
+      <c r="E55" s="47"/>
+      <c r="G55" s="64"/>
       <c r="H55" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="I55" s="72"/>
-      <c r="J55" s="68"/>
+      <c r="I55" s="4"/>
+      <c r="J55" s="5"/>
     </row>
     <row r="56" spans="2:10" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B56" s="42" t="s">
+      <c r="B56" s="60" t="s">
         <v>18</v>
       </c>
       <c r="C56" s="21" t="s">
         <v>61</v>
       </c>
-      <c r="D56" s="79"/>
-      <c r="E56" s="77"/>
+      <c r="D56" s="21"/>
+      <c r="E56" s="48"/>
     </row>
     <row r="57" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B57" s="43"/>
+      <c r="B57" s="61"/>
       <c r="C57" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="D57" s="65"/>
-      <c r="E57" s="66"/>
-      <c r="G57" s="47" t="s">
+      <c r="D57" s="2"/>
+      <c r="E57" s="3"/>
+      <c r="G57" s="65" t="s">
         <v>40</v>
       </c>
       <c r="H57" s="9" t="s">
         <v>61</v>
       </c>
-      <c r="I57" s="63"/>
-      <c r="J57" s="64"/>
+      <c r="I57" s="9"/>
+      <c r="J57" s="42"/>
     </row>
     <row r="58" spans="2:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B58" s="44"/>
+      <c r="B58" s="62"/>
       <c r="C58" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="D58" s="74"/>
-      <c r="E58" s="76"/>
-      <c r="G58" s="43"/>
+      <c r="D58" s="6"/>
+      <c r="E58" s="47"/>
+      <c r="G58" s="61"/>
       <c r="H58" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="I58" s="70"/>
-      <c r="J58" s="66"/>
+      <c r="I58" s="13"/>
+      <c r="J58" s="3"/>
     </row>
     <row r="59" spans="2:10" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B59" s="45" t="s">
+      <c r="B59" s="63" t="s">
         <v>19</v>
       </c>
       <c r="C59" s="13" t="s">
         <v>61</v>
       </c>
-      <c r="D59" s="70"/>
-      <c r="E59" s="71"/>
-      <c r="G59" s="44"/>
+      <c r="D59" s="13"/>
+      <c r="E59" s="44"/>
+      <c r="G59" s="62"/>
       <c r="H59" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="I59" s="74"/>
-      <c r="J59" s="76"/>
+      <c r="I59" s="6"/>
+      <c r="J59" s="47"/>
     </row>
     <row r="60" spans="2:10" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="B60" s="43"/>
+      <c r="B60" s="61"/>
       <c r="C60" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="D60" s="73"/>
-      <c r="E60" s="66"/>
-      <c r="G60" s="42" t="s">
+      <c r="D60" s="45"/>
+      <c r="E60" s="3"/>
+      <c r="G60" s="60" t="s">
         <v>41</v>
       </c>
       <c r="H60" s="21" t="s">
         <v>61</v>
       </c>
-      <c r="I60" s="79"/>
-      <c r="J60" s="77"/>
+      <c r="I60" s="21"/>
+      <c r="J60" s="48"/>
     </row>
     <row r="61" spans="2:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B61" s="46"/>
+      <c r="B61" s="64"/>
       <c r="C61" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="D61" s="72"/>
-      <c r="E61" s="68"/>
-      <c r="G61" s="43"/>
+      <c r="D61" s="4"/>
+      <c r="E61" s="5"/>
+      <c r="G61" s="61"/>
       <c r="H61" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="I61" s="65"/>
-      <c r="J61" s="66"/>
+      <c r="I61" s="2"/>
+      <c r="J61" s="3"/>
     </row>
     <row r="62" spans="2:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="D62" s="69"/>
-      <c r="E62" s="69"/>
-      <c r="G62" s="44"/>
+      <c r="G62" s="62"/>
       <c r="H62" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="I62" s="74"/>
-      <c r="J62" s="76"/>
+      <c r="I62" s="6"/>
+      <c r="J62" s="47"/>
     </row>
     <row r="63" spans="2:10" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="B63" s="47" t="s">
+      <c r="B63" s="65" t="s">
         <v>20</v>
       </c>
       <c r="C63" s="9" t="s">
         <v>61</v>
       </c>
-      <c r="D63" s="89"/>
-      <c r="E63" s="64"/>
-      <c r="G63" s="42" t="s">
+      <c r="D63" s="58"/>
+      <c r="E63" s="42"/>
+      <c r="G63" s="60" t="s">
         <v>42</v>
       </c>
       <c r="H63" s="21" t="s">
         <v>61</v>
       </c>
-      <c r="I63" s="79"/>
-      <c r="J63" s="77"/>
+      <c r="I63" s="21"/>
+      <c r="J63" s="48"/>
     </row>
     <row r="64" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B64" s="43"/>
+      <c r="B64" s="61"/>
       <c r="C64" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="D64" s="65"/>
-      <c r="E64" s="66"/>
-      <c r="G64" s="43"/>
+      <c r="D64" s="2"/>
+      <c r="E64" s="3"/>
+      <c r="G64" s="61"/>
       <c r="H64" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="I64" s="65"/>
-      <c r="J64" s="66"/>
+      <c r="I64" s="2"/>
+      <c r="J64" s="3"/>
     </row>
     <row r="65" spans="2:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B65" s="44"/>
+      <c r="B65" s="62"/>
       <c r="C65" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="D65" s="74"/>
-      <c r="E65" s="76"/>
-      <c r="G65" s="44"/>
+      <c r="D65" s="6"/>
+      <c r="E65" s="47"/>
+      <c r="G65" s="62"/>
       <c r="H65" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="I65" s="74"/>
-      <c r="J65" s="76"/>
+      <c r="I65" s="6"/>
+      <c r="J65" s="47"/>
     </row>
     <row r="66" spans="2:10" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="B66" s="42" t="s">
+      <c r="B66" s="60" t="s">
         <v>21</v>
       </c>
       <c r="C66" s="21" t="s">
         <v>61</v>
       </c>
-      <c r="D66" s="79"/>
-      <c r="E66" s="77"/>
-      <c r="G66" s="45" t="s">
+      <c r="D66" s="21"/>
+      <c r="E66" s="48"/>
+      <c r="G66" s="63" t="s">
         <v>43</v>
       </c>
       <c r="H66" s="13" t="s">
         <v>61</v>
       </c>
-      <c r="I66" s="70"/>
-      <c r="J66" s="71"/>
+      <c r="I66" s="13"/>
+      <c r="J66" s="44"/>
     </row>
     <row r="67" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B67" s="43"/>
+      <c r="B67" s="61"/>
       <c r="C67" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="D67" s="65"/>
-      <c r="E67" s="66"/>
-      <c r="G67" s="43"/>
+      <c r="D67" s="2"/>
+      <c r="E67" s="3"/>
+      <c r="G67" s="61"/>
       <c r="H67" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="I67" s="65"/>
-      <c r="J67" s="66"/>
+      <c r="I67" s="2"/>
+      <c r="J67" s="3"/>
     </row>
     <row r="68" spans="2:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B68" s="44"/>
+      <c r="B68" s="62"/>
       <c r="C68" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="D68" s="74"/>
-      <c r="E68" s="76"/>
-      <c r="G68" s="46"/>
+      <c r="D68" s="6"/>
+      <c r="E68" s="47"/>
+      <c r="G68" s="64"/>
       <c r="H68" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="I68" s="72"/>
-      <c r="J68" s="68"/>
+      <c r="I68" s="4"/>
+      <c r="J68" s="5"/>
     </row>
     <row r="69" spans="2:10" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B69" s="42" t="s">
+      <c r="B69" s="60" t="s">
         <v>22</v>
       </c>
       <c r="C69" s="21" t="s">
         <v>61</v>
       </c>
-      <c r="D69" s="79"/>
-      <c r="E69" s="77"/>
+      <c r="D69" s="21"/>
+      <c r="E69" s="48"/>
     </row>
     <row r="70" spans="2:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B70" s="43"/>
+      <c r="B70" s="61"/>
       <c r="C70" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="D70" s="65"/>
-      <c r="E70" s="66"/>
-      <c r="G70" s="48" t="s">
+      <c r="D70" s="2"/>
+      <c r="E70" s="3"/>
+      <c r="G70" s="66" t="s">
         <v>72</v>
       </c>
-      <c r="H70" s="49"/>
-      <c r="I70" s="49"/>
-      <c r="J70" s="50"/>
+      <c r="H70" s="67"/>
+      <c r="I70" s="67"/>
+      <c r="J70" s="68"/>
     </row>
     <row r="71" spans="2:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B71" s="44"/>
+      <c r="B71" s="62"/>
       <c r="C71" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="D71" s="74"/>
-      <c r="E71" s="76"/>
+      <c r="D71" s="6"/>
+      <c r="E71" s="47"/>
     </row>
     <row r="72" spans="2:10" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B72" s="42" t="s">
+      <c r="B72" s="60" t="s">
         <v>23</v>
       </c>
       <c r="C72" s="21" t="s">
         <v>61</v>
       </c>
-      <c r="D72" s="63"/>
-      <c r="E72" s="77"/>
+      <c r="D72" s="9"/>
+      <c r="E72" s="48"/>
       <c r="G72" s="14" t="s">
         <v>44</v>
       </c>
@@ -2607,19 +2593,19 @@
       </c>
     </row>
     <row r="73" spans="2:10" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="B73" s="43"/>
+      <c r="B73" s="61"/>
       <c r="C73" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="D73" s="65"/>
-      <c r="E73" s="66"/>
+      <c r="D73" s="2"/>
+      <c r="E73" s="3"/>
       <c r="G73" s="20" t="s">
         <v>74</v>
       </c>
       <c r="H73" s="27" t="s">
         <v>63</v>
       </c>
-      <c r="I73" s="65" t="s">
+      <c r="I73" s="2" t="s">
         <v>56</v>
       </c>
       <c r="J73" s="17" t="s">
@@ -2627,12 +2613,12 @@
       </c>
     </row>
     <row r="74" spans="2:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B74" s="44"/>
+      <c r="B74" s="62"/>
       <c r="C74" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="D74" s="70"/>
-      <c r="E74" s="76"/>
+      <c r="D74" s="13"/>
+      <c r="E74" s="47"/>
       <c r="G74" s="18" t="s">
         <v>75</v>
       </c>
@@ -2645,14 +2631,14 @@
       <c r="J74" s="3"/>
     </row>
     <row r="75" spans="2:10" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B75" s="42" t="s">
+      <c r="B75" s="60" t="s">
         <v>24</v>
       </c>
       <c r="C75" s="21" t="s">
         <v>61</v>
       </c>
-      <c r="D75" s="79"/>
-      <c r="E75" s="77"/>
+      <c r="D75" s="21"/>
+      <c r="E75" s="48"/>
       <c r="G75" s="36" t="s">
         <v>76</v>
       </c>
@@ -2665,24 +2651,24 @@
       <c r="J75" s="5"/>
     </row>
     <row r="76" spans="2:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B76" s="43"/>
+      <c r="B76" s="61"/>
       <c r="C76" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="D76" s="65"/>
-      <c r="E76" s="66"/>
+      <c r="D76" s="2"/>
+      <c r="E76" s="3"/>
       <c r="G76" s="38"/>
       <c r="H76" s="38"/>
       <c r="I76" s="38"/>
       <c r="J76" s="38"/>
     </row>
     <row r="77" spans="2:10" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B77" s="44"/>
+      <c r="B77" s="62"/>
       <c r="C77" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="D77" s="74"/>
-      <c r="E77" s="76"/>
+      <c r="D77" s="6"/>
+      <c r="E77" s="47"/>
       <c r="G77" s="37" t="s">
         <v>77</v>
       </c>
@@ -2697,14 +2683,14 @@
       </c>
     </row>
     <row r="78" spans="2:10" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="B78" s="45" t="s">
+      <c r="B78" s="63" t="s">
         <v>25</v>
       </c>
       <c r="C78" s="13" t="s">
         <v>61</v>
       </c>
-      <c r="D78" s="70"/>
-      <c r="E78" s="71"/>
+      <c r="D78" s="13"/>
+      <c r="E78" s="44"/>
       <c r="G78" s="18" t="s">
         <v>78</v>
       </c>
@@ -2717,12 +2703,12 @@
       <c r="J78" s="3"/>
     </row>
     <row r="79" spans="2:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B79" s="43"/>
+      <c r="B79" s="61"/>
       <c r="C79" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="D79" s="65"/>
-      <c r="E79" s="66"/>
+      <c r="D79" s="2"/>
+      <c r="E79" s="3"/>
       <c r="G79" s="19" t="s">
         <v>79</v>
       </c>
@@ -2735,12 +2721,12 @@
       <c r="J79" s="5"/>
     </row>
     <row r="80" spans="2:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B80" s="46"/>
+      <c r="B80" s="64"/>
       <c r="C80" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="D80" s="72"/>
-      <c r="E80" s="68"/>
+      <c r="D80" s="4"/>
+      <c r="E80" s="5"/>
     </row>
   </sheetData>
   <mergeCells count="40">
@@ -2786,7 +2772,7 @@
     <mergeCell ref="G70:J70"/>
   </mergeCells>
   <pageMargins left="0.31496062992125984" right="0.11811023622047245" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
-  <pageSetup paperSize="9" scale="40" orientation="landscape" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
+  <pageSetup paperSize="9" scale="93" fitToHeight="0" orientation="landscape" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
   <headerFooter>
     <oddHeader>&amp;C&amp;"Calibri"&amp;10&amp;K000000 UNCLASSIFIED&amp;1#_x000D_</oddHeader>
     <oddFooter>&amp;C_x000D_&amp;1#&amp;"Calibri"&amp;10&amp;K000000 UNCLASSIFIED</oddFooter>

</xml_diff>